<commit_message>
Added Maximum R to SNCImport page.
Also added to CSV download and IsoCheck chart.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56CA879A-FD19-47DA-A6AC-895764C41FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39AF678-A737-4E02-9F60-7C3561389EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-345" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19230" yWindow="2940" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="133">
   <si>
     <t>machine id</t>
   </si>
@@ -614,6 +614,9 @@
   </si>
   <si>
     <t>Gantry Flex (mm)</t>
+  </si>
+  <si>
+    <t>Maximum R (mm)</t>
   </si>
 </sst>
 </file>
@@ -3229,7 +3232,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C888577F-D905-495E-A65E-9EC6EA2BB2E5}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:C12"/>
+  <dimension ref="B2:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
@@ -3333,6 +3336,15 @@
       <c r="C12" s="34">
         <f>Collimator!L2</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" s="34">
+        <f>MAX(Data!I3:I13)</f>
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Maximum R Table 0 to spreadsheets.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39AF678-A737-4E02-9F60-7C3561389EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A375CB0D-C387-433F-AF2F-3E7CCD7826A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19230" yWindow="2940" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-345" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="134">
   <si>
     <t>machine id</t>
   </si>
@@ -617,6 +617,9 @@
   </si>
   <si>
     <t>Maximum R (mm)</t>
+  </si>
+  <si>
+    <t>Maximum R Table 0 (mm)</t>
   </si>
 </sst>
 </file>
@@ -3232,7 +3235,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C888577F-D905-495E-A65E-9EC6EA2BB2E5}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:C13"/>
+  <dimension ref="B2:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
@@ -3345,6 +3348,15 @@
       <c r="C13" s="34">
         <f>MAX(Data!I3:I13)</f>
         <v>-1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="33" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="34">
+        <f>_xlfn.MAXIFS(Preprocess!F3:I13, Preprocess!C3:F13, 0)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correctly calculate IsoCheck SNCImport values.
Add them instead of subtracting.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umhealth-my.sharepoint.com/personal/irrer_med_umich_edu/Documents/tmp/WLExcel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A375CB0D-C387-433F-AF2F-3E7CCD7826A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{A375CB0D-C387-433F-AF2F-3E7CCD7826A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AD950DD-1DF5-44BF-A7DA-54D8C9DE1BD8}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-345" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <definedName name="solver_eng" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="5" hidden="1">1</definedName>
@@ -72,6 +73,7 @@
     <definedName name="solver_neg" localSheetId="4" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="4" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="5" hidden="1">2147483647</definedName>
@@ -79,6 +81,7 @@
     <definedName name="solver_num" localSheetId="4" hidden="1">4</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_num" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="4" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="5" hidden="1">1</definedName>
@@ -86,6 +89,7 @@
     <definedName name="solver_opt" localSheetId="4" hidden="1">Collimator!$L$2</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">Data!$B$3</definedName>
     <definedName name="solver_opt" localSheetId="5" hidden="1">Report!$K$4</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">SNCImport!$B$6</definedName>
     <definedName name="solver_pre" localSheetId="3" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="4" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="5" hidden="1">0.000001</definedName>
@@ -149,14 +153,17 @@
     <definedName name="solver_typ" localSheetId="4" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_typ" localSheetId="5" hidden="1">1</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="4" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="5" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="4" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="5" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -512,12 +519,6 @@
     <t>CBCT - Gantry Iso Z (mm)</t>
   </si>
   <si>
-    <t>Table - Gantry Iso X (mm)</t>
-  </si>
-  <si>
-    <t>Table - Gantry Iso Z (mm)</t>
-  </si>
-  <si>
     <t>Col-Gantry misalignment (mm)</t>
   </si>
   <si>
@@ -620,6 +621,12 @@
   </si>
   <si>
     <t>Maximum R Table 0 (mm)</t>
+  </si>
+  <si>
+    <t>Table + Gantry Iso X (mm)</t>
+  </si>
+  <si>
+    <t>Table + Gantry Iso Z (mm)</t>
   </si>
 </sst>
 </file>
@@ -1358,6 +1365,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1365,7 +1373,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1705,6 +1712,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1712,7 +1720,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2937,6 +2944,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -3271,25 +3282,25 @@
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="33" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
       <c r="C5" s="34" t="e">
-        <f>Analysis!V5-Analysis!V$4</f>
+        <f>Analysis!V5+Analysis!V$4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="33" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
       <c r="C6" s="34" t="e">
-        <f>Analysis!X5-Analysis!X$4</f>
+        <f>Analysis!X5+Analysis!X$4</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C7" s="34" t="str">
         <f>Analysis!O3</f>
@@ -3298,7 +3309,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C8" s="34" t="e">
         <f>Analysis!P3</f>
@@ -3307,7 +3318,7 @@
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="33" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C9" s="34" t="str">
         <f>Analysis!T1</f>
@@ -3316,7 +3327,7 @@
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="33" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C10" s="34">
         <f>SQRT(Analysis!R12)</f>
@@ -3325,7 +3336,7 @@
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="33" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C11" s="34">
         <f>Analysis!O8</f>
@@ -3334,7 +3345,7 @@
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="33" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C12" s="34">
         <f>Collimator!L2</f>
@@ -3343,7 +3354,7 @@
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="33" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C13" s="34">
         <f>MAX(Data!I3:I13)</f>
@@ -3352,7 +3363,7 @@
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C14" s="34">
         <f>_xlfn.MAXIFS(Preprocess!F3:I13, Preprocess!C3:F13, 0)</f>
@@ -3395,13 +3406,13 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B1" s="38" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C1" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D1" s="38"/>
       <c r="E1" s="38"/>
@@ -3494,7 +3505,7 @@
         <v>21</v>
       </c>
       <c r="W2" s="38" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="X2" s="38" t="s">
         <v>97</v>
@@ -3505,13 +3516,13 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D3" s="38">
         <v>-1</v>
@@ -3568,27 +3579,27 @@
         <v>-1</v>
       </c>
       <c r="V3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y3" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D4" s="38">
         <v>-1</v>
@@ -3645,27 +3656,27 @@
         <v>-1</v>
       </c>
       <c r="V4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D5" s="38">
         <v>-1</v>
@@ -3722,27 +3733,27 @@
         <v>-1</v>
       </c>
       <c r="V5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y5" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D6" s="38">
         <v>-1</v>
@@ -3799,27 +3810,27 @@
         <v>-1</v>
       </c>
       <c r="V6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y6" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D7" s="38">
         <v>-1</v>
@@ -3876,27 +3887,27 @@
         <v>-1</v>
       </c>
       <c r="V7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y7" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D8" s="38">
         <v>-1</v>
@@ -3953,27 +3964,27 @@
         <v>-1</v>
       </c>
       <c r="V8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y8" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D9" s="38">
         <v>-1</v>
@@ -4030,27 +4041,27 @@
         <v>-1</v>
       </c>
       <c r="V9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D10" s="38">
         <v>-1</v>
@@ -4107,27 +4118,27 @@
         <v>-1</v>
       </c>
       <c r="V10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y10" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D11" s="38">
         <v>-1</v>
@@ -4184,27 +4195,27 @@
         <v>-1</v>
       </c>
       <c r="V11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y11" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D12" s="38">
         <v>-1</v>
@@ -4261,27 +4272,27 @@
         <v>-1</v>
       </c>
       <c r="V12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y12" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D13" s="38">
         <v>-1</v>
@@ -4338,16 +4349,16 @@
         <v>-1</v>
       </c>
       <c r="V13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="W13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="X13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="Y13" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
@@ -4488,7 +4499,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
@@ -6329,13 +6340,13 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="N6" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="O6" s="34" t="s">
         <v>112</v>
-      </c>
-      <c r="N6" s="34" t="s">
-        <v>113</v>
-      </c>
-      <c r="O6" s="34" t="s">
-        <v>114</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1" t="e">
@@ -6450,7 +6461,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="Q8" s="1" t="e">
         <f>-(F8-I$8)</f>
@@ -6622,7 +6633,7 @@
         <v>0</v>
       </c>
       <c r="S12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7064,7 +7075,7 @@
     <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H2" s="48" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I2" s="48"/>
       <c r="J2" s="48"/>
@@ -7074,12 +7085,12 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E3" s="22"/>
       <c r="F3" s="22" t="s">
@@ -7095,13 +7106,13 @@
         <v>33</v>
       </c>
       <c r="J3" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="L3" s="22" t="s">
         <v>116</v>
-      </c>
-      <c r="K3" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="L3" s="22" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -7514,7 +7525,7 @@
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="3:6" x14ac:dyDescent="0.25">
@@ -7522,7 +7533,7 @@
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="3:6" x14ac:dyDescent="0.25">
@@ -7538,7 +7549,7 @@
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="3:6" x14ac:dyDescent="0.25">
@@ -7554,7 +7565,7 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated instructions on spreadsheets.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate_11_Beams.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umhealth-my.sharepoint.com/personal/irrer_med_umich_edu/Documents/tmp/WLExcel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\tmp\aqaExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{A375CB0D-C387-433F-AF2F-3E7CCD7826A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AD950DD-1DF5-44BF-A7DA-54D8C9DE1BD8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80931850-81B2-401E-9994-56459919E5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -208,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="134">
   <si>
     <t>machine id</t>
   </si>
@@ -611,9 +611,6 @@
     <t>Winston-Lutz Field Data</t>
   </si>
   <si>
-    <t>To re-calculate spreadsheet in Excel, use CTRL-ALT-F9 and then run the solver on each of the Analysis and Collimator sheets.</t>
-  </si>
-  <si>
     <t>Gantry Flex (mm)</t>
   </si>
   <si>
@@ -627,6 +624,12 @@
   </si>
   <si>
     <t>Table + Gantry Iso Z (mm)</t>
+  </si>
+  <si>
+    <t>To re-calculate spreadsheet in Excel:
+    1: CTRL-ALT-F9 to calculate values
+    2: Set Excel's Solver to use "Evolutionary" (not "GRG Nonlinear")
+    3: Run the solver on each of the Analysis and Collimator sheets</t>
   </si>
 </sst>
 </file>
@@ -913,7 +916,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1014,6 +1017,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2944,10 +2958,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -3246,14 +3256,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C888577F-D905-495E-A65E-9EC6EA2BB2E5}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="B2:C14"/>
+  <dimension ref="B2:M14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
     <col min="3" max="3" width="8.85546875" style="22"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>100</v>
       </c>
@@ -3262,7 +3272,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="33" t="s">
         <v>101</v>
       </c>
@@ -3271,7 +3281,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="33" t="s">
         <v>102</v>
       </c>
@@ -3280,34 +3290,63 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="33" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C5" s="34" t="e">
         <f>Analysis!V5+Analysis!V$4</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E5" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="49"/>
+      <c r="M5" s="49"/>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="33" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C6" s="34" t="e">
         <f>Analysis!X5+Analysis!X$4</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C7" s="34" t="str">
         <f>Analysis!O3</f>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+      <c r="M7" s="49"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
         <v>103</v>
       </c>
@@ -3315,8 +3354,17 @@
         <f>Analysis!P3</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="33" t="s">
         <v>104</v>
       </c>
@@ -3325,7 +3373,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="33" t="s">
         <v>106</v>
       </c>
@@ -3334,7 +3382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="33" t="s">
         <v>107</v>
       </c>
@@ -3343,7 +3391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="33" t="s">
         <v>108</v>
       </c>
@@ -3352,18 +3400,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="33" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C13" s="34">
         <f>MAX(Data!I3:I13)</f>
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="33" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C14" s="34">
         <f>_xlfn.MAXIFS(Preprocess!F3:I13, Preprocess!C3:F13, 0)</f>
@@ -3372,6 +3420,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="E5:M8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4449,11 +4500,13 @@
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
       <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="42"/>
-      <c r="J17" s="42"/>
-      <c r="K17" s="42"/>
+      <c r="G17" s="52" t="s">
+        <v>133</v>
+      </c>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="51"/>
       <c r="L17" s="42"/>
       <c r="M17" s="42"/>
       <c r="N17" s="42"/>
@@ -4469,10 +4522,22 @@
       <c r="X17" s="42"/>
       <c r="Y17" s="42"/>
     </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="G18" s="51"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="51"/>
+      <c r="K18" s="51"/>
+    </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>52</v>
       </c>
+      <c r="G19" s="51"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -4484,6 +4549,11 @@
       <c r="C20" t="s">
         <v>55</v>
       </c>
+      <c r="G20" s="51"/>
+      <c r="H20" s="51"/>
+      <c r="I20" s="51"/>
+      <c r="J20" s="51"/>
+      <c r="K20" s="51"/>
     </row>
     <row r="21" spans="1:25" ht="21" x14ac:dyDescent="0.35">
       <c r="A21">
@@ -4498,9 +4568,7 @@
         <f t="shared" ref="C21" si="0">10*(C24-C23)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="41" t="s">
-        <v>128</v>
-      </c>
+      <c r="G21" s="41"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="39">
@@ -4532,6 +4600,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="G17:K20"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>